<commit_message>
Contraste con fuentes oficiales: cotización 2026, IRPF Aragón, inflación, factura electrónica, Verifactu y Anexo IV
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V4goTpBqBm77qbsNTgtkTF
</commit_message>
<xml_diff>
--- a/Modelo_financiero_Flujo.xlsx
+++ b/Modelo_financiero_Flujo.xlsx
@@ -897,10 +897,10 @@
         <v>4722.394907974109</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>25258.72105031152</v>
+        <v>25129.30060031152</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>47498.16329357418</v>
+        <v>46773.28038180168</v>
       </c>
     </row>
     <row r="8">
@@ -913,10 +913,10 @@
         <v>6242.122005206335</v>
       </c>
       <c r="C8" s="8" t="n">
-        <v>25822.26271697819</v>
+        <v>25692.84226697818</v>
       </c>
       <c r="D8" s="8" t="n">
-        <v>57820.03829357418</v>
+        <v>57095.15538180168</v>
       </c>
     </row>
     <row r="9">
@@ -945,10 +945,10 @@
         <v>6072.099462314975</v>
       </c>
       <c r="C10" s="6" t="n">
-        <v>34452.92556933349</v>
+        <v>34343.40186933349</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>70054.2084428223</v>
+        <v>69487.63824749729</v>
       </c>
     </row>
     <row r="11">
@@ -977,10 +977,10 @@
         <v>5472.099462314975</v>
       </c>
       <c r="C12" s="8" t="n">
-        <v>23052.92556933349</v>
+        <v>22943.40186933349</v>
       </c>
       <c r="D12" s="8" t="n">
-        <v>44254.2084428223</v>
+        <v>43687.63824749729</v>
       </c>
     </row>
     <row r="13">
@@ -1025,10 +1025,10 @@
         <v>770.0225428913586</v>
       </c>
       <c r="C15" s="6" t="n">
-        <v>2679.155023034104</v>
+        <v>2672.278573034105</v>
       </c>
       <c r="D15" s="6" t="n">
-        <v>3414.809849132276</v>
+        <v>3379.827139359776</v>
       </c>
     </row>
     <row r="16">
@@ -1041,10 +1041,10 @@
         <v>0</v>
       </c>
       <c r="C16" s="6" t="n">
-        <v>90.18212461059284</v>
+        <v>77.16182461058906</v>
       </c>
       <c r="D16" s="6" t="n">
-        <v>1733.092203957296</v>
+        <v>1609.762197282294</v>
       </c>
     </row>
     <row r="17">
@@ -1057,10 +1057,10 @@
         <v>770.0225428913586</v>
       </c>
       <c r="C17" s="8" t="n">
-        <v>2769.337147644697</v>
+        <v>2749.440397644694</v>
       </c>
       <c r="D17" s="8" t="n">
-        <v>13565.82985075189</v>
+        <v>13407.51713430439</v>
       </c>
     </row>
     <row r="18">
@@ -1073,10 +1073,10 @@
         <v>6242.122005206333</v>
       </c>
       <c r="C18" s="8" t="n">
-        <v>25822.26271697819</v>
+        <v>25692.84226697819</v>
       </c>
       <c r="D18" s="8" t="n">
-        <v>57820.03829357419</v>
+        <v>57095.15538180168</v>
       </c>
     </row>
   </sheetData>
@@ -1147,10 +1147,10 @@
         <v>-5008.412605870877</v>
       </c>
       <c r="C3" s="6" t="n">
-        <v>-7305.996135030544</v>
+        <v>-7486.681935030543</v>
       </c>
       <c r="D3" s="6" t="n">
-        <v>-17806.03934977379</v>
+        <v>-18639.88871504879</v>
       </c>
     </row>
     <row r="4">
@@ -1163,10 +1163,10 @@
         <v>-770.7314529428633</v>
       </c>
       <c r="C4" s="6" t="n">
-        <v>-5846.388430659896</v>
+        <v>-5825.759080659895</v>
       </c>
       <c r="D4" s="6" t="n">
-        <v>-8438.341155522587</v>
+        <v>-8358.068677520088</v>
       </c>
     </row>
     <row r="5">
@@ -1179,10 +1179,10 @@
         <v>-776.7536589524022</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>-4459.418312119524</v>
+        <v>-4428.782312119525</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>-7546.695897703944</v>
+        <v>-7388.58147220394</v>
       </c>
     </row>
     <row r="6">
@@ -1195,10 +1195,10 @@
         <v>5897.144907974108</v>
       </c>
       <c r="C6" s="8" t="n">
-        <v>31880.82614233741</v>
+        <v>31751.4056923374</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>42741.51444560035</v>
+        <v>42146.05198382785</v>
       </c>
     </row>
     <row r="7">
@@ -1323,10 +1323,10 @@
         <v>4722.394907974109</v>
       </c>
       <c r="C14" s="8" t="n">
-        <v>25258.72105031152</v>
+        <v>25129.30060031152</v>
       </c>
       <c r="D14" s="8" t="n">
-        <v>47498.16329357418</v>
+        <v>46773.28038180168</v>
       </c>
     </row>
   </sheetData>
@@ -1390,10 +1390,10 @@
         <v>733.7904711304418</v>
       </c>
       <c r="D2" s="6" t="n">
-        <v>9533.199418678792</v>
+        <v>9403.778968678791</v>
       </c>
       <c r="E2" s="6" t="n">
-        <v>7482.675944543055</v>
+        <v>6949.26482218556</v>
       </c>
     </row>
     <row r="3">
@@ -1409,10 +1409,10 @@
         <v>-7257.654528869559</v>
       </c>
       <c r="D3" s="6" t="n">
-        <v>-6449.690581321209</v>
+        <v>-6579.11103132121</v>
       </c>
       <c r="E3" s="6" t="n">
-        <v>-8500.214055456945</v>
+        <v>-9033.625177814441</v>
       </c>
     </row>
     <row r="4">
@@ -1428,10 +1428,10 @@
         <v>3855.833495592202</v>
       </c>
       <c r="D4" s="6" t="n">
-        <v>21963.54326136578</v>
+        <v>21834.12281136577</v>
       </c>
       <c r="E4" s="6" t="n">
-        <v>27267.18666232774</v>
+        <v>26693.28152526274</v>
       </c>
     </row>
     <row r="5">
@@ -1447,10 +1447,10 @@
         <v>-4135.611504407799</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>5980.653261365775</v>
+        <v>5851.23281136577</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>11284.29666232774</v>
+        <v>10710.39152526274</v>
       </c>
     </row>
     <row r="6">
@@ -1466,10 +1466,10 @@
         <v>6147.394907974109</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>31336.32614233741</v>
+        <v>31206.90569233741</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>30672.28201697382</v>
+        <v>30076.81955520132</v>
       </c>
     </row>
     <row r="7">
@@ -1485,10 +1485,10 @@
         <v>-1844.050092025892</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>15353.43614233741</v>
+        <v>15224.01569233741</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>14689.39201697382</v>
+        <v>14093.92955520132</v>
       </c>
     </row>
     <row r="9">
@@ -1521,13 +1521,13 @@
         </is>
       </c>
       <c r="B10" s="6" t="n">
-        <v>9866.277935625005</v>
+        <v>9417.691010428984</v>
       </c>
       <c r="C10" s="6" t="n">
-        <v>34988.86068353354</v>
+        <v>34513.648286351</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>46307.59867030993</v>
+        <v>45818.2119822044</v>
       </c>
       <c r="E10" s="6" t="n"/>
     </row>
@@ -1538,13 +1538,13 @@
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>35516.45677528961</v>
+        <v>32537.62887705847</v>
       </c>
       <c r="C11" s="6" t="n">
-        <v>154487.0632170893</v>
+        <v>151289.5260846831</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>181957.9049420453</v>
+        <v>178643.9361342003</v>
       </c>
       <c r="E11" s="6" t="n"/>
     </row>
@@ -1555,13 +1555,13 @@
         </is>
       </c>
       <c r="B12" s="3" t="n">
-        <v>1.237459138111535</v>
+        <v>1.210355956947313</v>
       </c>
       <c r="C12" s="3" t="n">
-        <v>2.894162828820328</v>
+        <v>2.880633784535879</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>3.817861485244056</v>
+        <v>3.806892067313734</v>
       </c>
       <c r="E12" s="3" t="n"/>
     </row>
@@ -1572,7 +1572,7 @@
         </is>
       </c>
       <c r="B13" s="9" t="n">
-        <v>1.227254191769525</v>
+        <v>1.230381800347009</v>
       </c>
       <c r="C13" s="9" t="n">
         <v>0.7521720020626986</v>
@@ -1589,7 +1589,7 @@
         </is>
       </c>
       <c r="B14" s="9" t="n">
-        <v>1.313821357532728</v>
+        <v>1.318140355400157</v>
       </c>
       <c r="C14" s="9" t="n">
         <v>0.8649978023721033</v>
@@ -1606,13 +1606,13 @@
         </is>
       </c>
       <c r="B15" s="6" t="n">
-        <v>-19677.17534784669</v>
+        <v>-20125.76227304271</v>
       </c>
       <c r="C15" s="6" t="n">
-        <v>5445.407400061853</v>
+        <v>4970.195002879305</v>
       </c>
       <c r="D15" s="6" t="n">
-        <v>16764.14538683824</v>
+        <v>16274.7586987327</v>
       </c>
       <c r="E15" s="6" t="n"/>
     </row>
@@ -1624,10 +1624,10 @@
       </c>
       <c r="B16" s="3" t="n"/>
       <c r="C16" s="3" t="n">
-        <v>0.5434244654427329</v>
+        <v>0.5149215702417351</v>
       </c>
       <c r="D16" s="3" t="n">
-        <v>1.418684266884273</v>
+        <v>1.398095734537629</v>
       </c>
       <c r="E16" s="3" t="n"/>
     </row>
@@ -3128,22 +3128,22 @@
         <v>150.7499929061046</v>
       </c>
       <c r="AF12" s="6" t="n">
-        <v>182.0640840989513</v>
+        <v>183.7598865989513</v>
       </c>
       <c r="AG12" s="6" t="n">
-        <v>207.3170264583711</v>
+        <v>210.3694709583711</v>
       </c>
       <c r="AH12" s="6" t="n">
-        <v>231.5951719944279</v>
+        <v>236.0042584944279</v>
       </c>
       <c r="AI12" s="6" t="n">
-        <v>256.0667869237012</v>
+        <v>261.8325154237012</v>
       </c>
       <c r="AJ12" s="6" t="n">
-        <v>280.6526976175824</v>
+        <v>287.7750681175824</v>
       </c>
       <c r="AK12" s="6" t="n">
-        <v>305.3061307324011</v>
+        <v>313.7851432324011</v>
       </c>
     </row>
     <row r="13">
@@ -3225,40 +3225,40 @@
         <v>80</v>
       </c>
       <c r="Z13" s="6" t="n">
-        <v>440</v>
+        <v>452.94</v>
       </c>
       <c r="AA13" s="6" t="n">
-        <v>440</v>
+        <v>452.94</v>
       </c>
       <c r="AB13" s="6" t="n">
-        <v>440</v>
+        <v>452.94</v>
       </c>
       <c r="AC13" s="6" t="n">
-        <v>440</v>
+        <v>452.94</v>
       </c>
       <c r="AD13" s="6" t="n">
-        <v>440</v>
+        <v>452.94</v>
       </c>
       <c r="AE13" s="6" t="n">
-        <v>440</v>
+        <v>452.94</v>
       </c>
       <c r="AF13" s="6" t="n">
-        <v>440</v>
+        <v>452.94</v>
       </c>
       <c r="AG13" s="6" t="n">
-        <v>440</v>
+        <v>452.94</v>
       </c>
       <c r="AH13" s="6" t="n">
-        <v>440</v>
+        <v>452.94</v>
       </c>
       <c r="AI13" s="6" t="n">
-        <v>440</v>
+        <v>452.94</v>
       </c>
       <c r="AJ13" s="6" t="n">
-        <v>440</v>
+        <v>452.94</v>
       </c>
       <c r="AK13" s="6" t="n">
-        <v>440</v>
+        <v>452.94</v>
       </c>
     </row>
     <row r="14">
@@ -3304,76 +3304,76 @@
         <v>195</v>
       </c>
       <c r="N14" s="6" t="n">
-        <v>195</v>
+        <v>202.215</v>
       </c>
       <c r="O14" s="6" t="n">
-        <v>195</v>
+        <v>202.215</v>
       </c>
       <c r="P14" s="6" t="n">
-        <v>195</v>
+        <v>202.215</v>
       </c>
       <c r="Q14" s="6" t="n">
-        <v>195</v>
+        <v>202.215</v>
       </c>
       <c r="R14" s="6" t="n">
-        <v>195</v>
+        <v>202.215</v>
       </c>
       <c r="S14" s="6" t="n">
-        <v>195</v>
+        <v>202.215</v>
       </c>
       <c r="T14" s="6" t="n">
-        <v>195</v>
+        <v>202.215</v>
       </c>
       <c r="U14" s="6" t="n">
-        <v>195</v>
+        <v>202.215</v>
       </c>
       <c r="V14" s="6" t="n">
-        <v>195</v>
+        <v>202.215</v>
       </c>
       <c r="W14" s="6" t="n">
-        <v>195</v>
+        <v>202.215</v>
       </c>
       <c r="X14" s="6" t="n">
-        <v>195</v>
+        <v>202.215</v>
       </c>
       <c r="Y14" s="6" t="n">
-        <v>195</v>
+        <v>202.215</v>
       </c>
       <c r="Z14" s="6" t="n">
-        <v>195</v>
+        <v>209.696955</v>
       </c>
       <c r="AA14" s="6" t="n">
-        <v>195</v>
+        <v>209.696955</v>
       </c>
       <c r="AB14" s="6" t="n">
-        <v>195</v>
+        <v>209.696955</v>
       </c>
       <c r="AC14" s="6" t="n">
-        <v>195</v>
+        <v>209.696955</v>
       </c>
       <c r="AD14" s="6" t="n">
-        <v>195</v>
+        <v>209.696955</v>
       </c>
       <c r="AE14" s="6" t="n">
-        <v>195</v>
+        <v>209.696955</v>
       </c>
       <c r="AF14" s="6" t="n">
-        <v>195</v>
+        <v>209.696955</v>
       </c>
       <c r="AG14" s="6" t="n">
-        <v>195</v>
+        <v>209.696955</v>
       </c>
       <c r="AH14" s="6" t="n">
-        <v>195</v>
+        <v>209.696955</v>
       </c>
       <c r="AI14" s="6" t="n">
-        <v>195</v>
+        <v>209.696955</v>
       </c>
       <c r="AJ14" s="6" t="n">
-        <v>195</v>
+        <v>209.696955</v>
       </c>
       <c r="AK14" s="6" t="n">
-        <v>195</v>
+        <v>209.696955</v>
       </c>
     </row>
     <row r="15">
@@ -3419,76 +3419,76 @@
         <v>50</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>150</v>
+        <v>155.55</v>
       </c>
       <c r="O15" s="6" t="n">
-        <v>150</v>
+        <v>155.55</v>
       </c>
       <c r="P15" s="6" t="n">
-        <v>150</v>
+        <v>155.55</v>
       </c>
       <c r="Q15" s="6" t="n">
-        <v>150</v>
+        <v>155.55</v>
       </c>
       <c r="R15" s="6" t="n">
-        <v>150</v>
+        <v>155.55</v>
       </c>
       <c r="S15" s="6" t="n">
-        <v>150</v>
+        <v>155.55</v>
       </c>
       <c r="T15" s="6" t="n">
-        <v>150</v>
+        <v>155.55</v>
       </c>
       <c r="U15" s="6" t="n">
-        <v>150</v>
+        <v>155.55</v>
       </c>
       <c r="V15" s="6" t="n">
-        <v>150</v>
+        <v>155.55</v>
       </c>
       <c r="W15" s="6" t="n">
-        <v>150</v>
+        <v>155.55</v>
       </c>
       <c r="X15" s="6" t="n">
-        <v>150</v>
+        <v>155.55</v>
       </c>
       <c r="Y15" s="6" t="n">
-        <v>150</v>
+        <v>155.55</v>
       </c>
       <c r="Z15" s="6" t="n">
-        <v>300</v>
+        <v>322.6107</v>
       </c>
       <c r="AA15" s="6" t="n">
-        <v>300</v>
+        <v>322.6107</v>
       </c>
       <c r="AB15" s="6" t="n">
-        <v>300</v>
+        <v>322.6107</v>
       </c>
       <c r="AC15" s="6" t="n">
-        <v>300</v>
+        <v>322.6107</v>
       </c>
       <c r="AD15" s="6" t="n">
-        <v>300</v>
+        <v>322.6107</v>
       </c>
       <c r="AE15" s="6" t="n">
-        <v>300</v>
+        <v>322.6107</v>
       </c>
       <c r="AF15" s="6" t="n">
-        <v>300</v>
+        <v>322.6107</v>
       </c>
       <c r="AG15" s="6" t="n">
-        <v>300</v>
+        <v>322.6107</v>
       </c>
       <c r="AH15" s="6" t="n">
-        <v>300</v>
+        <v>322.6107</v>
       </c>
       <c r="AI15" s="6" t="n">
-        <v>300</v>
+        <v>322.6107</v>
       </c>
       <c r="AJ15" s="6" t="n">
-        <v>300</v>
+        <v>322.6107</v>
       </c>
       <c r="AK15" s="6" t="n">
-        <v>300</v>
+        <v>322.6107</v>
       </c>
     </row>
     <row r="16">
@@ -3588,22 +3588,22 @@
         <v>0</v>
       </c>
       <c r="AF16" s="6" t="n">
-        <v>150</v>
+        <v>161.30535</v>
       </c>
       <c r="AG16" s="6" t="n">
-        <v>150</v>
+        <v>161.30535</v>
       </c>
       <c r="AH16" s="6" t="n">
-        <v>150</v>
+        <v>161.30535</v>
       </c>
       <c r="AI16" s="6" t="n">
-        <v>150</v>
+        <v>161.30535</v>
       </c>
       <c r="AJ16" s="6" t="n">
-        <v>150</v>
+        <v>161.30535</v>
       </c>
       <c r="AK16" s="6" t="n">
-        <v>150</v>
+        <v>161.30535</v>
       </c>
     </row>
     <row r="17">
@@ -3879,76 +3879,76 @@
         <v>2430.833495592201</v>
       </c>
       <c r="N19" s="8" t="n">
-        <v>1712.510322627646</v>
+        <v>1697.453172627646</v>
       </c>
       <c r="O19" s="8" t="n">
-        <v>2266.50524108925</v>
+        <v>2236.39094108925</v>
       </c>
       <c r="P19" s="8" t="n">
-        <v>2734.632526870199</v>
+        <v>2697.1200768702</v>
       </c>
       <c r="Q19" s="8" t="n">
-        <v>2906.070475437867</v>
+        <v>2860.377325437868</v>
       </c>
       <c r="R19" s="8" t="n">
-        <v>4062.926859777912</v>
+        <v>4002.176559777913</v>
       </c>
       <c r="S19" s="8" t="n">
-        <v>5567.215183271929</v>
+        <v>5499.06673327193</v>
       </c>
       <c r="T19" s="8" t="n">
-        <v>5891.05064156862</v>
+        <v>5814.721491568622</v>
       </c>
       <c r="U19" s="8" t="n">
-        <v>7601.135644424094</v>
+        <v>7509.749344424096</v>
       </c>
       <c r="V19" s="8" t="n">
-        <v>8695.547106622074</v>
+        <v>8596.762656622077</v>
       </c>
       <c r="W19" s="8" t="n">
-        <v>9563.547883351835</v>
+        <v>9456.582733351839</v>
       </c>
       <c r="X19" s="8" t="n">
-        <v>12181.94748787817</v>
+        <v>12059.92518787818</v>
       </c>
       <c r="Y19" s="8" t="n">
-        <v>13594.37675695797</v>
+        <v>13464.95630695798</v>
       </c>
       <c r="Z19" s="8" t="n">
-        <v>21352.58115620239</v>
+        <v>21172.7462681524</v>
       </c>
       <c r="AA19" s="8" t="n">
-        <v>21066.63504146912</v>
+        <v>20829.50926536912</v>
       </c>
       <c r="AB19" s="8" t="n">
-        <v>19644.11881522618</v>
+        <v>19379.85074407619</v>
       </c>
       <c r="AC19" s="8" t="n">
-        <v>18823.74073698896</v>
+        <v>18523.31147693897</v>
       </c>
       <c r="AD19" s="8" t="n">
-        <v>19083.92128645875</v>
+        <v>18726.20113835876</v>
       </c>
       <c r="AE19" s="8" t="n">
-        <v>18771.31613158876</v>
+        <v>18399.47398843877</v>
       </c>
       <c r="AF19" s="8" t="n">
-        <v>20599.81570328683</v>
+        <v>20176.08097671184</v>
       </c>
       <c r="AG19" s="8" t="n">
-        <v>23862.50906094235</v>
+        <v>23364.11051497237</v>
       </c>
       <c r="AH19" s="8" t="n">
-        <v>25684.82132199604</v>
+        <v>25148.88068951105</v>
       </c>
       <c r="AI19" s="8" t="n">
-        <v>26537.65248739419</v>
+        <v>25953.9400715592</v>
       </c>
       <c r="AJ19" s="8" t="n">
-        <v>30329.57158024129</v>
+        <v>29666.2707345513</v>
       </c>
       <c r="AK19" s="8" t="n">
-        <v>32428.72364557455</v>
+        <v>31725.39805850956</v>
       </c>
     </row>
   </sheetData>
@@ -4102,7 +4102,7 @@
         <v>-913.4313000715401</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>-2273.47427947941</v>
+        <v>-2303.99872447941</v>
       </c>
     </row>
     <row r="9">
@@ -4118,7 +4118,7 @@
         <v>30401.9887046978</v>
       </c>
       <c r="D9" s="8" t="n">
-        <v>55821.47768581459</v>
+        <v>55790.95324081459</v>
       </c>
     </row>
     <row r="10">
@@ -4134,7 +4134,7 @@
         <v>-960</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>-5280</v>
+        <v>-5435.28</v>
       </c>
     </row>
     <row r="11">
@@ -4147,10 +4147,10 @@
         <v>-2340</v>
       </c>
       <c r="C11" s="6" t="n">
-        <v>-2340</v>
+        <v>-2426.58</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>-2340</v>
+        <v>-2516.36346</v>
       </c>
     </row>
     <row r="12">
@@ -4163,10 +4163,10 @@
         <v>-600</v>
       </c>
       <c r="C12" s="6" t="n">
-        <v>-1800</v>
+        <v>-1866.6</v>
       </c>
       <c r="D12" s="6" t="n">
-        <v>-3600</v>
+        <v>-3871.328399999999</v>
       </c>
     </row>
     <row r="13">
@@ -4182,7 +4182,7 @@
         <v>0</v>
       </c>
       <c r="D13" s="6" t="n">
-        <v>-900</v>
+        <v>-967.8320999999999</v>
       </c>
     </row>
     <row r="14">
@@ -4211,10 +4211,10 @@
         <v>3670.661837579344</v>
       </c>
       <c r="C15" s="8" t="n">
-        <v>25301.9887046978</v>
+        <v>25148.8087046978</v>
       </c>
       <c r="D15" s="8" t="n">
-        <v>43701.47768581459</v>
+        <v>43000.14928081459</v>
       </c>
     </row>
     <row r="16">
@@ -4243,10 +4243,10 @@
         <v>3541.495170912678</v>
       </c>
       <c r="C17" s="8" t="n">
-        <v>25069.69703803114</v>
+        <v>24916.51703803114</v>
       </c>
       <c r="D17" s="8" t="n">
-        <v>41459.81101914793</v>
+        <v>40758.48261414793</v>
       </c>
     </row>
     <row r="18">
@@ -4275,10 +4275,10 @@
         <v>3541.495170912678</v>
       </c>
       <c r="C19" s="8" t="n">
-        <v>25069.69703803114</v>
+        <v>24916.51703803114</v>
       </c>
       <c r="D19" s="8" t="n">
-        <v>40863.75138204717</v>
+        <v>40162.42297704717</v>
       </c>
     </row>
     <row r="20">
@@ -4291,10 +4291,10 @@
         <v>0</v>
       </c>
       <c r="C20" s="6" t="n">
-        <v>-4210.001155838873</v>
+        <v>-4166.344855838873</v>
       </c>
       <c r="D20" s="6" t="n">
-        <v>-8919.125511357453</v>
+        <v>-8659.634001507453</v>
       </c>
     </row>
     <row r="21">
@@ -4307,10 +4307,10 @@
         <v>3541.495170912678</v>
       </c>
       <c r="C21" s="8" t="n">
-        <v>20859.69588219226</v>
+        <v>20750.17218219226</v>
       </c>
       <c r="D21" s="8" t="n">
-        <v>31944.62587068972</v>
+        <v>31502.78897553972</v>
       </c>
     </row>
   </sheetData>
@@ -4429,7 +4429,7 @@
         <v>708.2990341825354</v>
       </c>
       <c r="C6" s="6" t="n">
-        <v>803.9382517673548</v>
+        <v>816.9585517673559</v>
       </c>
       <c r="D6" s="6" t="n">
         <v>0</v>
@@ -4445,10 +4445,10 @@
         <v>2430.833495592201</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>13594.37675695797</v>
+        <v>13464.95630695798</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>32428.72364557455</v>
+        <v>31725.39805850956</v>
       </c>
     </row>
     <row r="8">
@@ -4461,10 +4461,10 @@
         <v>3484.96586310807</v>
       </c>
       <c r="C8" s="8" t="n">
-        <v>14961.85667539199</v>
+        <v>14845.456525392</v>
       </c>
       <c r="D8" s="8" t="n">
-        <v>42750.59864557455</v>
+        <v>42047.27305850956</v>
       </c>
     </row>
     <row r="9">
@@ -4493,10 +4493,10 @@
         <v>3541.495170912678</v>
       </c>
       <c r="C10" s="6" t="n">
-        <v>24401.19105310494</v>
+        <v>24291.66735310494</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>56345.81692379466</v>
+        <v>55794.45632864466</v>
       </c>
     </row>
     <row r="11">
@@ -4525,10 +4525,10 @@
         <v>2941.495170912678</v>
       </c>
       <c r="C12" s="8" t="n">
-        <v>13001.19105310494</v>
+        <v>12891.66735310494</v>
       </c>
       <c r="D12" s="8" t="n">
-        <v>30545.81692379466</v>
+        <v>29994.45632864466</v>
       </c>
     </row>
     <row r="13">
@@ -4573,10 +4573,10 @@
         <v>543.4706921953932</v>
       </c>
       <c r="C15" s="6" t="n">
-        <v>1960.665622287056</v>
+        <v>1953.789172287056</v>
       </c>
       <c r="D15" s="6" t="n">
-        <v>3040.478689169565</v>
+        <v>3007.739526104565</v>
       </c>
     </row>
     <row r="16">
@@ -4592,7 +4592,7 @@
         <v>0</v>
       </c>
       <c r="D16" s="6" t="n">
-        <v>746.3752349480201</v>
+        <v>627.1494060980185</v>
       </c>
     </row>
     <row r="17">
@@ -4605,10 +4605,10 @@
         <v>543.4706921953932</v>
       </c>
       <c r="C17" s="8" t="n">
-        <v>1960.665622287056</v>
+        <v>1953.789172287056</v>
       </c>
       <c r="D17" s="8" t="n">
-        <v>12204.7817217799</v>
+        <v>12052.8167298649</v>
       </c>
     </row>
     <row r="18">
@@ -4621,10 +4621,10 @@
         <v>3484.965863108071</v>
       </c>
       <c r="C18" s="8" t="n">
-        <v>14961.85667539199</v>
+        <v>14845.45652539199</v>
       </c>
       <c r="D18" s="8" t="n">
-        <v>42750.59864557456</v>
+        <v>42047.27305850956</v>
       </c>
     </row>
   </sheetData>
@@ -4695,10 +4695,10 @@
         <v>-4960.849251118849</v>
       </c>
       <c r="C3" s="6" t="n">
-        <v>-6948.651873086564</v>
+        <v>-7129.337673086564</v>
       </c>
       <c r="D3" s="6" t="n">
-        <v>-16777.36351527084</v>
+        <v>-17583.86559132085</v>
       </c>
     </row>
     <row r="4">
@@ -4711,10 +4711,10 @@
         <v>-455.218293696269</v>
       </c>
       <c r="C4" s="6" t="n">
-        <v>-4129.322697894877</v>
+        <v>-4108.693347894877</v>
       </c>
       <c r="D4" s="6" t="n">
-        <v>-6812.297247138555</v>
+        <v>-6732.986289153554</v>
       </c>
     </row>
     <row r="5">
@@ -4727,10 +4727,10 @@
         <v>-370.5652299405734</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>-3209.63273322338</v>
+        <v>-3178.996733223381</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>-5557.564042099731</v>
+        <v>-5404.278061099731</v>
       </c>
     </row>
     <row r="6">
@@ -4743,10 +4743,10 @@
         <v>3605.583495592201</v>
       </c>
       <c r="C6" s="8" t="n">
-        <v>22508.04326136578</v>
+        <v>22378.62281136578</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>39336.41909095426</v>
+        <v>38762.51395388926</v>
       </c>
     </row>
     <row r="7">
@@ -4871,10 +4871,10 @@
         <v>2430.833495592201</v>
       </c>
       <c r="C14" s="8" t="n">
-        <v>13594.37675695797</v>
+        <v>13464.95630695798</v>
       </c>
       <c r="D14" s="8" t="n">
-        <v>32428.72364557455</v>
+        <v>31725.39805850956</v>
       </c>
     </row>
   </sheetData>
@@ -5028,7 +5028,7 @@
         <v>-475.0030709646414</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>-1158.254349909176</v>
+        <v>-1173.516572409176</v>
       </c>
     </row>
     <row r="9">
@@ -5044,7 +5044,7 @@
         <v>16401.86832667812</v>
       </c>
       <c r="D9" s="8" t="n">
-        <v>29323.70231070255</v>
+        <v>29308.44008820255</v>
       </c>
     </row>
     <row r="10">
@@ -5060,7 +5060,7 @@
         <v>-960</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>-3492</v>
+        <v>-3594.72</v>
       </c>
     </row>
     <row r="11">
@@ -5073,10 +5073,10 @@
         <v>-2340</v>
       </c>
       <c r="C11" s="6" t="n">
-        <v>-2340</v>
+        <v>-2426.58</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>-2340</v>
+        <v>-2516.36346</v>
       </c>
     </row>
     <row r="12">
@@ -5089,10 +5089,10 @@
         <v>-600</v>
       </c>
       <c r="C12" s="6" t="n">
-        <v>-1800</v>
+        <v>-1866.6</v>
       </c>
       <c r="D12" s="6" t="n">
-        <v>-3600</v>
+        <v>-3871.328399999999</v>
       </c>
     </row>
     <row r="13">
@@ -5108,7 +5108,7 @@
         <v>0</v>
       </c>
       <c r="D13" s="6" t="n">
-        <v>-900</v>
+        <v>-967.8320999999999</v>
       </c>
     </row>
     <row r="14">
@@ -5137,10 +5137,10 @@
         <v>324.7182592406807</v>
       </c>
       <c r="C15" s="8" t="n">
-        <v>11301.86832667812</v>
+        <v>11148.68832667812</v>
       </c>
       <c r="D15" s="8" t="n">
-        <v>18991.70231070255</v>
+        <v>18358.19612820255</v>
       </c>
     </row>
     <row r="16">
@@ -5169,10 +5169,10 @@
         <v>195.5515925740141</v>
       </c>
       <c r="C17" s="8" t="n">
-        <v>11069.57666001145</v>
+        <v>10916.39666001145</v>
       </c>
       <c r="D17" s="8" t="n">
-        <v>16750.03564403588</v>
+        <v>16116.52946153588</v>
       </c>
     </row>
     <row r="18">
@@ -5201,10 +5201,10 @@
         <v>195.5515925740141</v>
       </c>
       <c r="C19" s="8" t="n">
-        <v>11069.57666001145</v>
+        <v>10916.39666001145</v>
       </c>
       <c r="D19" s="8" t="n">
-        <v>16153.97600693512</v>
+        <v>15520.46982443512</v>
       </c>
     </row>
     <row r="20">
@@ -5217,10 +5217,10 @@
         <v>0</v>
       </c>
       <c r="C20" s="6" t="n">
-        <v>-943.5585871320675</v>
+        <v>-915.9095971320673</v>
       </c>
       <c r="D20" s="6" t="n">
-        <v>-1990.544029581207</v>
+        <v>-1846.104619971208</v>
       </c>
     </row>
     <row r="21">
@@ -5233,10 +5233,10 @@
         <v>195.5515925740141</v>
       </c>
       <c r="C21" s="8" t="n">
-        <v>10126.01807287939</v>
+        <v>10000.48706287939</v>
       </c>
       <c r="D21" s="8" t="n">
-        <v>14163.43197735391</v>
+        <v>13674.36520446392</v>
       </c>
     </row>
   </sheetData>
@@ -5355,10 +5355,10 @@
         <v>195.0641288204149</v>
       </c>
       <c r="C6" s="6" t="n">
-        <v>1270.356744870223</v>
+        <v>1267.369734870223</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>1240.251171805818</v>
+        <v>1257.989344915817</v>
       </c>
     </row>
     <row r="7">
@@ -5371,10 +5371,10 @@
         <v>-691.2095288695574</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>-1958.010110190767</v>
+        <v>-2087.430560190768</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>-2992.814407827176</v>
+        <v>-3655.645980184678</v>
       </c>
     </row>
     <row r="8">
@@ -5387,10 +5387,10 @@
         <v>-150.3120667158092</v>
       </c>
       <c r="C8" s="8" t="n">
-        <v>-124.1116986538775</v>
+        <v>-256.5191586538776</v>
       </c>
       <c r="D8" s="8" t="n">
-        <v>8569.311763978641</v>
+        <v>7924.218364731139</v>
       </c>
     </row>
     <row r="9">
@@ -5419,10 +5419,10 @@
         <v>195.5515925740141</v>
       </c>
       <c r="C10" s="6" t="n">
-        <v>10321.5696654534</v>
+        <v>10196.0386554534</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>24485.00164280731</v>
+        <v>23870.40385991731</v>
       </c>
     </row>
     <row r="11">
@@ -5451,10 +5451,10 @@
         <v>-404.4484074259858</v>
       </c>
       <c r="C12" s="8" t="n">
-        <v>-1078.4303345466</v>
+        <v>-1203.9613445466</v>
       </c>
       <c r="D12" s="8" t="n">
-        <v>-1314.99835719269</v>
+        <v>-1929.596140082685</v>
       </c>
     </row>
     <row r="13">
@@ -5499,10 +5499,10 @@
         <v>254.136340710176</v>
       </c>
       <c r="C15" s="6" t="n">
-        <v>954.3186358927242</v>
+        <v>947.4421858927242</v>
       </c>
       <c r="D15" s="6" t="n">
-        <v>1466.38232350901</v>
+        <v>1435.88670715151</v>
       </c>
     </row>
     <row r="16">
@@ -5531,10 +5531,10 @@
         <v>254.136340710176</v>
       </c>
       <c r="C17" s="8" t="n">
-        <v>954.3186358927242</v>
+        <v>947.4421858927242</v>
       </c>
       <c r="D17" s="8" t="n">
-        <v>9884.310121171326</v>
+        <v>9853.814504813825</v>
       </c>
     </row>
     <row r="18">
@@ -5547,10 +5547,10 @@
         <v>-150.3120667158098</v>
       </c>
       <c r="C18" s="8" t="n">
-        <v>-124.1116986538755</v>
+        <v>-256.519158653876</v>
       </c>
       <c r="D18" s="8" t="n">
-        <v>8569.311763978636</v>
+        <v>7924.218364731139</v>
       </c>
     </row>
   </sheetData>
@@ -5621,10 +5621,10 @@
         <v>-4899.195569954536</v>
       </c>
       <c r="C3" s="6" t="n">
-        <v>-6418.153715867214</v>
+        <v>-6598.839515867216</v>
       </c>
       <c r="D3" s="6" t="n">
-        <v>-13639.94740049086</v>
+        <v>-14375.42218731586</v>
       </c>
     </row>
     <row r="4">
@@ -5637,10 +5637,10 @@
         <v>-41.90449373036701</v>
       </c>
       <c r="C4" s="6" t="n">
-        <v>-1906.310053419856</v>
+        <v>-1885.680703419856</v>
       </c>
       <c r="D4" s="6" t="n">
-        <v>-1815.513797631249</v>
+        <v>-1737.164359663749</v>
       </c>
     </row>
     <row r="5">
@@ -5653,10 +5653,10 @@
         <v>-0</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>-1419.642604480879</v>
+        <v>-1389.00660448088</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>-994.5662767711099</v>
+        <v>-870.8520502711092</v>
       </c>
     </row>
     <row r="6">
@@ -5669,10 +5669,10 @@
         <v>483.5404711304436</v>
       </c>
       <c r="C6" s="8" t="n">
-        <v>10077.69941867879</v>
+        <v>9948.278968678793</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>19467.26790470128</v>
+        <v>18933.85678234378</v>
       </c>
     </row>
     <row r="7">
@@ -5797,10 +5797,10 @@
         <v>-691.2095288695574</v>
       </c>
       <c r="C14" s="8" t="n">
-        <v>-1958.010110190767</v>
+        <v>-2087.430560190768</v>
       </c>
       <c r="D14" s="8" t="n">
-        <v>-2992.814407827176</v>
+        <v>-3655.645980184678</v>
       </c>
     </row>
   </sheetData>
@@ -5954,7 +5954,7 @@
         <v>-1208.757136388879</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>-2875.685712952919</v>
+        <v>-2921.472380452919</v>
       </c>
     </row>
     <row r="9">
@@ -5970,7 +5970,7 @@
         <v>40921.05195620305</v>
       </c>
       <c r="D9" s="8" t="n">
-        <v>61925.69515057505</v>
+        <v>61879.90848307504</v>
       </c>
     </row>
     <row r="10">
@@ -5986,7 +5986,7 @@
         <v>-960</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>-5580</v>
+        <v>-5744.16</v>
       </c>
     </row>
     <row r="11">
@@ -5999,10 +5999,10 @@
         <v>-2340</v>
       </c>
       <c r="C11" s="6" t="n">
-        <v>-2340</v>
+        <v>-2426.58</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>-2340</v>
+        <v>-2516.36346</v>
       </c>
     </row>
     <row r="12">
@@ -6015,10 +6015,10 @@
         <v>-600</v>
       </c>
       <c r="C12" s="6" t="n">
-        <v>-1800</v>
+        <v>-1866.6</v>
       </c>
       <c r="D12" s="6" t="n">
-        <v>-3600</v>
+        <v>-3871.328399999999</v>
       </c>
     </row>
     <row r="13">
@@ -6034,7 +6034,7 @@
         <v>0</v>
       </c>
       <c r="D13" s="6" t="n">
-        <v>-900</v>
+        <v>-967.8320999999999</v>
       </c>
     </row>
     <row r="14">
@@ -6063,10 +6063,10 @@
         <v>6251.923789686771</v>
       </c>
       <c r="C15" s="8" t="n">
-        <v>35821.05195620305</v>
+        <v>35667.87195620305</v>
       </c>
       <c r="D15" s="8" t="n">
-        <v>49505.69515057505</v>
+        <v>48780.22452307504</v>
       </c>
     </row>
     <row r="16">
@@ -6095,10 +6095,10 @@
         <v>6122.757123020104</v>
       </c>
       <c r="C17" s="8" t="n">
-        <v>35588.76028953639</v>
+        <v>35435.58028953639</v>
       </c>
       <c r="D17" s="8" t="n">
-        <v>47264.02848390838</v>
+        <v>46538.55785640838</v>
       </c>
     </row>
     <row r="18">
@@ -6127,10 +6127,10 @@
         <v>6122.757123020104</v>
       </c>
       <c r="C19" s="8" t="n">
-        <v>35588.76028953639</v>
+        <v>35435.58028953639</v>
       </c>
       <c r="D19" s="8" t="n">
-        <v>46667.96884680763</v>
+        <v>45942.49821930762</v>
       </c>
     </row>
     <row r="20">
@@ -6143,10 +6143,10 @@
         <v>-50.65766070512859</v>
       </c>
       <c r="C20" s="6" t="n">
-        <v>-7207.934182517871</v>
+        <v>-7164.277882517868</v>
       </c>
       <c r="D20" s="6" t="n">
-        <v>-11066.68597331882</v>
+        <v>-10798.26184114382</v>
       </c>
     </row>
     <row r="21">
@@ -6159,10 +6159,10 @@
         <v>6072.099462314975</v>
       </c>
       <c r="C21" s="8" t="n">
-        <v>28380.82610701852</v>
+        <v>28271.30240701852</v>
       </c>
       <c r="D21" s="8" t="n">
-        <v>35601.2828734888</v>
+        <v>35144.2363781638</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Capítulo 8: mejora de la rentabilidad (LTV/CAC, VAN por línea, palancas, Montecarlo, autónomo frente a SL)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V4goTpBqBm77qbsNTgtkTF
</commit_message>
<xml_diff>
--- a/Modelo_financiero_Flujo.xlsx
+++ b/Modelo_financiero_Flujo.xlsx
@@ -19,6 +19,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Balance optimista" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash-flow optimista" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Valoración" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Palancas de mejora" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PyG plan mejorado" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Montecarlo" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1646,6 +1649,639 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="48" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Medida (acumulada)</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>VAN</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>VAN con coste de oportunidad</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Mejora del VAN c.o.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Escenario base</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="n">
+        <v>34513.648286351</v>
+      </c>
+      <c r="C2" s="6" t="n">
+        <v>4970.195002879305</v>
+      </c>
+      <c r="D2" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Actualización anual de precios con el IPC</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="n">
+        <v>37377.89572383671</v>
+      </c>
+      <c r="C3" s="6" t="n">
+        <v>7834.442440365011</v>
+      </c>
+      <c r="D3" s="6" t="n">
+        <v>2864.247437485706</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Estandarización del servicio (2 h por cliente desde el año 2)</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="n">
+        <v>38346.5358277437</v>
+      </c>
+      <c r="C4" s="6" t="n">
+        <v>8803.082544272002</v>
+      </c>
+      <c r="D4" s="6" t="n">
+        <v>968.6401039069906</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Talleres grupales para instituciones (1 al mes en el año 2 y 2 en el año 3)</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="n">
+        <v>43524.9288975226</v>
+      </c>
+      <c r="C5" s="6" t="n">
+        <v>13981.47561405091</v>
+      </c>
+      <c r="D5" s="6" t="n">
+        <v>5178.393069778904</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Acuerdo de derivación con gestorías (30 % de las altas)</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="n">
+        <v>44403.11231167564</v>
+      </c>
+      <c r="C6" s="6" t="n">
+        <v>14859.65902820394</v>
+      </c>
+      <c r="D6" s="6" t="n">
+        <v>878.1834141530362</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Herramienta no-code de 5.000 € sin microcrédito</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="n">
+        <v>48918.93169523693</v>
+      </c>
+      <c r="C7" s="6" t="n">
+        <v>19375.47841176525</v>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>4515.819383561304</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="48" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Cuenta de resultados</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Año 1</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Año 2</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Año 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Ingresos por setup</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="n">
+        <v>2800</v>
+      </c>
+      <c r="C2" s="6" t="n">
+        <v>6221.999999999999</v>
+      </c>
+      <c r="D2" s="6" t="n">
+        <v>7742.656799999999</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Ingresos por suscripción</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="n">
+        <v>5241.281053380045</v>
+      </c>
+      <c r="C3" s="6" t="n">
+        <v>20838.95054494581</v>
+      </c>
+      <c r="D3" s="6" t="n">
+        <v>40169.98439473286</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Ingresos por plantillas</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="6" t="n">
+        <v>2799.9</v>
+      </c>
+      <c r="D4" s="6" t="n">
+        <v>6290.908649999999</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Ingresos por cursos</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="6" t="n">
+        <v>2613.24</v>
+      </c>
+      <c r="D5" s="6" t="n">
+        <v>6323.169719999999</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Ingresos por la herramienta digital</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" s="6" t="n">
+        <v>3484.195559999999</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>IMPORTE NETO DE LA CIFRA DE NEGOCIOS</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="n">
+        <v>8293.281053380044</v>
+      </c>
+      <c r="C7" s="8" t="n">
+        <v>36125.09054494581</v>
+      </c>
+      <c r="D7" s="8" t="n">
+        <v>71111.12912473285</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Costes variables (comisiones, alojamiento)</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="n">
+        <v>-120.6192158007007</v>
+      </c>
+      <c r="C8" s="6" t="n">
+        <v>-947.2282581741871</v>
+      </c>
+      <c r="D8" s="6" t="n">
+        <v>-2467.884833320993</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>MARGEN DE CONTRIBUCIÓN</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="n">
+        <v>8172.661837579343</v>
+      </c>
+      <c r="C9" s="8" t="n">
+        <v>35177.86228677162</v>
+      </c>
+      <c r="D9" s="8" t="n">
+        <v>68643.24429141186</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Cuota de autónomos (RETA)</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="n">
+        <v>-960</v>
+      </c>
+      <c r="C10" s="6" t="n">
+        <v>-960</v>
+      </c>
+      <c r="D10" s="6" t="n">
+        <v>-6052.92</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Otros gastos fijos de explotación</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="n">
+        <v>-2340</v>
+      </c>
+      <c r="C11" s="6" t="n">
+        <v>-2426.58</v>
+      </c>
+      <c r="D11" s="6" t="n">
+        <v>-2516.36346</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Marketing</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="n">
+        <v>-600</v>
+      </c>
+      <c r="C12" s="6" t="n">
+        <v>-1866.6</v>
+      </c>
+      <c r="D12" s="6" t="n">
+        <v>-3871.328399999999</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Mantenimiento de la herramienta</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" s="6" t="n">
+        <v>-967.8320999999999</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Gastos de puesta en marcha</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="n">
+        <v>-350</v>
+      </c>
+      <c r="C14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>EBITDA</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="n">
+        <v>3922.661837579343</v>
+      </c>
+      <c r="C15" s="8" t="n">
+        <v>29924.68228677162</v>
+      </c>
+      <c r="D15" s="8" t="n">
+        <v>55234.80033141186</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Amortización del inmovilizado</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="n">
+        <v>-129.1666666666667</v>
+      </c>
+      <c r="C16" s="6" t="n">
+        <v>-232.2916666666666</v>
+      </c>
+      <c r="D16" s="6" t="n">
+        <v>-1075</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>RESULTADO DE EXPLOTACIÓN (EBIT)</t>
+        </is>
+      </c>
+      <c r="B17" s="8" t="n">
+        <v>3793.495170912677</v>
+      </c>
+      <c r="C17" s="8" t="n">
+        <v>29692.39062010495</v>
+      </c>
+      <c r="D17" s="8" t="n">
+        <v>54159.80033141186</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Gastos financieros</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="n">
+        <v>-0</v>
+      </c>
+      <c r="C18" s="6" t="n">
+        <v>-0</v>
+      </c>
+      <c r="D18" s="6" t="n">
+        <v>-0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>RESULTADO ANTES DE IMPUESTOS</t>
+        </is>
+      </c>
+      <c r="B19" s="8" t="n">
+        <v>3793.495170912677</v>
+      </c>
+      <c r="C19" s="8" t="n">
+        <v>29692.39062010495</v>
+      </c>
+      <c r="D19" s="8" t="n">
+        <v>54159.80033141186</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>IRPF imputable a la actividad (estimado)</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="6" t="n">
+        <v>-5527.468826729911</v>
+      </c>
+      <c r="D20" s="6" t="n">
+        <v>-13838.66362262239</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>RESULTADO NETO DISPONIBLE PARA EL TITULAR</t>
+        </is>
+      </c>
+      <c r="B21" s="8" t="n">
+        <v>3793.495170912677</v>
+      </c>
+      <c r="C21" s="8" t="n">
+        <v>24164.92179337504</v>
+      </c>
+      <c r="D21" s="8" t="n">
+        <v>40321.13670878948</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Ingresos por talleres</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="6" t="n">
+        <v>3111</v>
+      </c>
+      <c r="D22" s="6" t="n">
+        <v>6452.213999999998</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Ingresos por derivación a gestorías</t>
+        </is>
+      </c>
+      <c r="B23" s="6" t="n">
+        <v>252</v>
+      </c>
+      <c r="C23" s="6" t="n">
+        <v>540</v>
+      </c>
+      <c r="D23" s="6" t="n">
+        <v>647.9999999999999</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="48" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Indicador</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Plan base</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Plan mejorado</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Probabilidad VAN &gt; 0</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" s="3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Probabilidad VAN con coste de oportunidad &gt; 0</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="n">
+        <v>0.5705</v>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>0.9535</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>VAN c.o. percentil 5</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="n">
+        <v>-12029.46544851666</v>
+      </c>
+      <c r="C4" s="6" t="n">
+        <v>250.4302837658063</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>VAN c.o. mediana</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="n">
+        <v>1410.95589197782</v>
+      </c>
+      <c r="C5" s="6" t="n">
+        <v>14665.09591375303</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>VAN c.o. percentil 95</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="n">
+        <v>9855.222967951118</v>
+      </c>
+      <c r="C6" s="6" t="n">
+        <v>25807.86938377781</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>